<commit_message>
hnaya tmajt bzaf file exel  w9a3 lihom combine bach power query idmajhom f sheet wahda wn9dar ndir elihom analysis
</commit_message>
<xml_diff>
--- a/mergeFile/trade1.xlsx
+++ b/mergeFile/trade1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\mergeFile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8B3E04-B3E6-47A6-9FEA-7A39B6B50C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082C1127-68FD-4105-8A6B-67497A9354FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4F1D4521-0189-43F1-9026-999CE5ACD4D5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>pair</t>
   </si>
@@ -75,6 +75,24 @@
   </si>
   <si>
     <t>24-09-2027</t>
+  </si>
+  <si>
+    <t>us30</t>
+  </si>
+  <si>
+    <t>24-09-2028</t>
+  </si>
+  <si>
+    <t>A009</t>
+  </si>
+  <si>
+    <t>A010</t>
+  </si>
+  <si>
+    <t>gold</t>
+  </si>
+  <si>
+    <t>24-09-2029</t>
   </si>
 </sst>
 </file>
@@ -262,14 +280,6 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -369,6 +379,15 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -376,19 +395,18 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -404,14 +422,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0F4D8C93-ACD7-4D79-BC72-4E06D3A21B32}" name="trader1" displayName="trader1" ref="B3:F5" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="7" tableBorderDxfId="8" totalsRowBorderDxfId="6">
-  <autoFilter ref="B3:F5" xr:uid="{0F4D8C93-ACD7-4D79-BC72-4E06D3A21B32}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0F4D8C93-ACD7-4D79-BC72-4E06D3A21B32}" name="trader1" displayName="trader1" ref="B3:F7" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
+  <autoFilter ref="B3:F7" xr:uid="{0F4D8C93-ACD7-4D79-BC72-4E06D3A21B32}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{F3C2708F-22B0-4FF6-AA46-BB9C85A866A0}" name="tradeid" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{4BE9C31E-1CF8-4674-938D-07A74D0F42DE}" name="pair" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{0593F66D-E017-4282-B877-F0516D54B876}" name="profit" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{86FA1E7A-D9A1-4FB6-9467-6FFF7DFEA08F}" name="setup" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{0C69FD24-20D9-452A-99C2-547F5D8100B7}" name="date" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{F3C2708F-22B0-4FF6-AA46-BB9C85A866A0}" name="tradeid" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{4BE9C31E-1CF8-4674-938D-07A74D0F42DE}" name="pair" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{0593F66D-E017-4282-B877-F0516D54B876}" name="profit" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{86FA1E7A-D9A1-4FB6-9467-6FFF7DFEA08F}" name="setup" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{0C69FD24-20D9-452A-99C2-547F5D8100B7}" name="date" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -796,18 +814,38 @@
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="5"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="7"/>
+      <c r="B6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="13">
+        <v>738</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="5"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="7"/>
+      <c r="B7" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="13">
+        <v>-763</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="5"/>

</xml_diff>